<commit_message>
Updated Rate Build Up and Reports
</commit_message>
<xml_diff>
--- a/data/externalStats/File1/RPT_RPT1980057586629RA_externalStats.xlsx
+++ b/data/externalStats/File1/RPT_RPT1980057586629RA_externalStats.xlsx
@@ -2181,7 +2181,7 @@
         <v>11053681.77593989</v>
       </c>
       <c r="AI26" s="56" t="n">
-        <v>14824.51869790835</v>
+        <v>14824.51869790836</v>
       </c>
       <c r="AK26" s="123" t="n">
         <v>2</v>
@@ -3523,7 +3523,7 @@
         <v>1035027.547097453</v>
       </c>
       <c r="AI44" s="84" t="n">
-        <v>1651.013328294837</v>
+        <v>1651.013328294838</v>
       </c>
       <c r="AK44" s="126" t="n">
         <v>20</v>
@@ -3958,7 +3958,7 @@
         </is>
       </c>
       <c r="AG53" s="122" t="n">
-        <v>6254997.388832267</v>
+        <v>6254997.388832266</v>
       </c>
       <c r="AH53" s="56" t="n">
         <v>974.78778950125</v>
@@ -3992,7 +3992,7 @@
         <v>10902.85394682596</v>
       </c>
       <c r="L54" s="131" t="n">
-        <v>3100.939586379484</v>
+        <v>3100.939586379483</v>
       </c>
       <c r="M54" s="131" t="n">
         <v>0</v>
@@ -4001,19 +4001,19 @@
         <v>34480.29792294405</v>
       </c>
       <c r="P54" s="130" t="n">
-        <v>21660.72763903786</v>
+        <v>21660.72763903787</v>
       </c>
       <c r="Q54" s="131" t="n">
         <v>11377.65923837764</v>
       </c>
       <c r="R54" s="131" t="n">
-        <v>3422.487711428825</v>
+        <v>3422.487711428826</v>
       </c>
       <c r="S54" s="131" t="n">
         <v>0</v>
       </c>
       <c r="T54" s="132" t="n">
-        <v>36460.87458884433</v>
+        <v>36460.87458884434</v>
       </c>
       <c r="V54" s="130" t="n">
         <v>23326.03531108902</v>
@@ -4022,13 +4022,13 @@
         <v>12035.45165849652</v>
       </c>
       <c r="X54" s="131" t="n">
-        <v>3876.170523329414</v>
+        <v>3876.170523329415</v>
       </c>
       <c r="Y54" s="131" t="n">
         <v>0</v>
       </c>
       <c r="Z54" s="132" t="n">
-        <v>39237.65749291495</v>
+        <v>39237.65749291496</v>
       </c>
       <c r="AE54" s="121" t="n">
         <v>6</v>
@@ -4313,10 +4313,10 @@
         <v>2594.410828881019</v>
       </c>
       <c r="K58" s="131" t="n">
-        <v>985.1537316312742</v>
+        <v>985.1537316312744</v>
       </c>
       <c r="L58" s="131" t="n">
-        <v>255.8945333813836</v>
+        <v>255.8945333813835</v>
       </c>
       <c r="M58" s="131" t="n">
         <v>0</v>
@@ -4328,16 +4328,16 @@
         <v>2524.098090035488</v>
       </c>
       <c r="Q58" s="131" t="n">
-        <v>955.4907245728979</v>
+        <v>955.4907245728981</v>
       </c>
       <c r="R58" s="131" t="n">
-        <v>249.3325380336442</v>
+        <v>249.3325380336441</v>
       </c>
       <c r="S58" s="131" t="n">
         <v>0</v>
       </c>
       <c r="T58" s="132" t="n">
-        <v>3728.921352642029</v>
+        <v>3728.92135264203</v>
       </c>
       <c r="V58" s="130" t="n">
         <v>2448.763529811295</v>
@@ -4352,7 +4352,7 @@
         <v>0</v>
       </c>
       <c r="Z58" s="132" t="n">
-        <v>3615.028403056119</v>
+        <v>3615.02840305612</v>
       </c>
       <c r="AE58" s="121" t="n">
         <v>10</v>
@@ -4640,7 +4640,7 @@
         <v>32.36265349002131</v>
       </c>
       <c r="L62" s="131" t="n">
-        <v>5.262228230812023</v>
+        <v>5.262228230812022</v>
       </c>
       <c r="M62" s="131" t="n">
         <v>0</v>
@@ -4676,7 +4676,7 @@
         <v>0</v>
       </c>
       <c r="Z62" s="132" t="n">
-        <v>86.19003294722576</v>
+        <v>86.19003294722577</v>
       </c>
       <c r="AE62" s="121" t="n">
         <v>14</v>
@@ -4718,10 +4718,10 @@
         <v>5470.853056493306</v>
       </c>
       <c r="K63" s="131" t="n">
-        <v>1628.922856379853</v>
+        <v>1628.922856379852</v>
       </c>
       <c r="L63" s="131" t="n">
-        <v>579.4673615811294</v>
+        <v>579.4673615811298</v>
       </c>
       <c r="M63" s="131" t="n">
         <v>17013.70034841627</v>
@@ -4730,34 +4730,34 @@
         <v>24692.94362287056</v>
       </c>
       <c r="P63" s="130" t="n">
-        <v>5717.989908079238</v>
+        <v>5717.989908079231</v>
       </c>
       <c r="Q63" s="131" t="n">
         <v>1677.905544971887</v>
       </c>
       <c r="R63" s="131" t="n">
-        <v>603.0641618903842</v>
+        <v>603.0641618903837</v>
       </c>
       <c r="S63" s="131" t="n">
         <v>18677.29304011533</v>
       </c>
       <c r="T63" s="132" t="n">
-        <v>26676.25265505684</v>
+        <v>26676.25265505683</v>
       </c>
       <c r="V63" s="130" t="n">
-        <v>5996.295669644594</v>
+        <v>5996.295669644587</v>
       </c>
       <c r="W63" s="131" t="n">
-        <v>1742.154527729672</v>
+        <v>1742.154527729668</v>
       </c>
       <c r="X63" s="131" t="n">
-        <v>629.6630878851374</v>
+        <v>629.6630878851365</v>
       </c>
       <c r="Y63" s="131" t="n">
         <v>20543.90331686658</v>
       </c>
       <c r="Z63" s="132" t="n">
-        <v>28912.01660212599</v>
+        <v>28912.01660212598</v>
       </c>
       <c r="AE63" s="121" t="n">
         <v>15</v>
@@ -4771,7 +4771,7 @@
         <v>880391.1703553336</v>
       </c>
       <c r="AH63" s="56" t="n">
-        <v>2705.748534253711</v>
+        <v>2705.748534253712</v>
       </c>
     </row>
     <row r="64">
@@ -4852,7 +4852,7 @@
         <v>782128.8810255195</v>
       </c>
       <c r="AH64" s="56" t="n">
-        <v>797.2439270399999</v>
+        <v>797.24392704</v>
       </c>
     </row>
     <row r="65">
@@ -5017,7 +5017,7 @@
         </is>
       </c>
       <c r="AG66" s="122" t="n">
-        <v>490934.3341392858</v>
+        <v>490934.3341392857</v>
       </c>
       <c r="AH66" s="56" t="n">
         <v>2589.08465126051</v>
@@ -5132,13 +5132,13 @@
         <v>13549.2931883271</v>
       </c>
       <c r="L68" s="143" t="n">
-        <v>3941.563709572809</v>
+        <v>3941.563709572808</v>
       </c>
       <c r="M68" s="143" t="n">
         <v>17013.70034841627</v>
       </c>
       <c r="N68" s="144" t="n">
-        <v>78603.70350424443</v>
+        <v>78603.70350424442</v>
       </c>
       <c r="P68" s="142" t="n">
         <v>29955.58714387762</v>
@@ -5156,7 +5156,7 @@
         <v>84055.34524985497</v>
       </c>
       <c r="V68" s="142" t="n">
-        <v>31822.07038902595</v>
+        <v>31822.07038902594</v>
       </c>
       <c r="W68" s="143" t="n">
         <v>14731.87121800636</v>
@@ -5403,34 +5403,34 @@
         <v>116</v>
       </c>
       <c r="J72" s="130" t="n">
-        <v>60.36280720546834</v>
+        <v>60.36280720546836</v>
       </c>
       <c r="K72" s="131" t="n">
-        <v>17.22156077641948</v>
+        <v>17.22156077641947</v>
       </c>
       <c r="L72" s="131" t="n">
-        <v>11.88892922423182</v>
+        <v>11.88892922423181</v>
       </c>
       <c r="M72" s="131" t="n">
         <v>0</v>
       </c>
       <c r="N72" s="132" t="n">
-        <v>89.47329720611963</v>
+        <v>89.47329720611964</v>
       </c>
       <c r="P72" s="130" t="n">
-        <v>54.7544447970989</v>
+        <v>54.75444479709888</v>
       </c>
       <c r="Q72" s="131" t="n">
         <v>13.17974339598205</v>
       </c>
       <c r="R72" s="131" t="n">
-        <v>9.1285333020486</v>
+        <v>9.128533302048602</v>
       </c>
       <c r="S72" s="131" t="n">
         <v>0</v>
       </c>
       <c r="T72" s="132" t="n">
-        <v>77.06272149512955</v>
+        <v>77.06272149512952</v>
       </c>
       <c r="V72" s="130" t="n">
         <v>48.60500608217873</v>
@@ -5445,7 +5445,7 @@
         <v>0</v>
       </c>
       <c r="Z72" s="132" t="n">
-        <v>63.00658003928496</v>
+        <v>63.00658003928495</v>
       </c>
     </row>
     <row r="73">
@@ -5540,7 +5540,7 @@
         <v>144.1175339064627</v>
       </c>
       <c r="K74" s="131" t="n">
-        <v>15.89356319143109</v>
+        <v>15.89356319143108</v>
       </c>
       <c r="L74" s="131" t="n">
         <v>0</v>
@@ -5552,7 +5552,7 @@
         <v>168.6890429822031</v>
       </c>
       <c r="P74" s="130" t="n">
-        <v>137.9660640772048</v>
+        <v>137.9660640772047</v>
       </c>
       <c r="Q74" s="131" t="n">
         <v>12.14013438652261</v>
@@ -5567,7 +5567,7 @@
         <v>158.2054900284876</v>
       </c>
       <c r="V74" s="130" t="n">
-        <v>129.0017416528368</v>
+        <v>129.0017416528367</v>
       </c>
       <c r="W74" s="131" t="n">
         <v>8.002227321906959</v>
@@ -5677,7 +5677,7 @@
         <v>28.64956631726437</v>
       </c>
       <c r="L76" s="131" t="n">
-        <v>8.426940306992982</v>
+        <v>8.42694030699298</v>
       </c>
       <c r="M76" s="131" t="n">
         <v>0</v>
@@ -5692,7 +5692,7 @@
         <v>22.65146691033027</v>
       </c>
       <c r="R76" s="131" t="n">
-        <v>6.653565310419796</v>
+        <v>6.653565310419798</v>
       </c>
       <c r="S76" s="131" t="n">
         <v>0</v>
@@ -5701,7 +5701,7 @@
         <v>129.5250851430111</v>
       </c>
       <c r="V76" s="130" t="n">
-        <v>91.34566034189018</v>
+        <v>91.34566034189017</v>
       </c>
       <c r="W76" s="131" t="n">
         <v>15.38658979934373</v>
@@ -6006,13 +6006,13 @@
         <v>2397</v>
       </c>
       <c r="J81" s="130" t="n">
-        <v>0</v>
+        <v>-5.684341886080801e-14</v>
       </c>
       <c r="K81" s="131" t="n">
-        <v>-7.105427357601002e-15</v>
+        <v>0</v>
       </c>
       <c r="L81" s="131" t="n">
-        <v>0</v>
+        <v>3.552713678800501e-15</v>
       </c>
       <c r="M81" s="131" t="n">
         <v>2668.418392338495</v>
@@ -6021,22 +6021,22 @@
         <v>2668.418392338495</v>
       </c>
       <c r="P81" s="130" t="n">
-        <v>0</v>
+        <v>5.684341886080801e-14</v>
       </c>
       <c r="Q81" s="131" t="n">
         <v>0</v>
       </c>
       <c r="R81" s="131" t="n">
-        <v>0</v>
+        <v>-1.77635683940025e-15</v>
       </c>
       <c r="S81" s="131" t="n">
-        <v>2915.32683331261</v>
+        <v>2915.326833312611</v>
       </c>
       <c r="T81" s="132" t="n">
-        <v>2915.32683331261</v>
+        <v>2915.326833312611</v>
       </c>
       <c r="V81" s="130" t="n">
-        <v>-5.684341886080801e-14</v>
+        <v>0</v>
       </c>
       <c r="W81" s="131" t="n">
         <v>-7.105427357601002e-15</v>
@@ -6372,7 +6372,7 @@
         <v>2923.426124877371</v>
       </c>
       <c r="T86" s="144" t="n">
-        <v>4942.501101949607</v>
+        <v>4942.501101949608</v>
       </c>
       <c r="V86" s="142" t="n">
         <v>268.9524080769056</v>
@@ -6608,22 +6608,22 @@
         <v>32117</v>
       </c>
       <c r="J90" s="130" t="n">
-        <v>20536.86719694408</v>
+        <v>20536.86719694407</v>
       </c>
       <c r="K90" s="131" t="n">
         <v>10920.07550760238</v>
       </c>
       <c r="L90" s="131" t="n">
-        <v>3112.828515603716</v>
+        <v>3112.828515603715</v>
       </c>
       <c r="M90" s="131" t="n">
         <v>0</v>
       </c>
       <c r="N90" s="132" t="n">
-        <v>34569.77122015017</v>
+        <v>34569.77122015016</v>
       </c>
       <c r="P90" s="130" t="n">
-        <v>21715.48208383496</v>
+        <v>21715.48208383497</v>
       </c>
       <c r="Q90" s="131" t="n">
         <v>11390.83898177362</v>
@@ -6635,22 +6635,22 @@
         <v>0</v>
       </c>
       <c r="T90" s="132" t="n">
-        <v>36537.93731033946</v>
+        <v>36537.93731033947</v>
       </c>
       <c r="V90" s="130" t="n">
         <v>23374.6403171712</v>
       </c>
       <c r="W90" s="131" t="n">
-        <v>12044.16326397683</v>
+        <v>12044.16326397684</v>
       </c>
       <c r="X90" s="131" t="n">
-        <v>3881.860491806206</v>
+        <v>3881.860491806207</v>
       </c>
       <c r="Y90" s="131" t="n">
         <v>0</v>
       </c>
       <c r="Z90" s="132" t="n">
-        <v>39300.66407295423</v>
+        <v>39300.66407295424</v>
       </c>
     </row>
     <row r="91">
@@ -6745,7 +6745,7 @@
         <v>144.1175339064627</v>
       </c>
       <c r="K92" s="131" t="n">
-        <v>15.89356319143109</v>
+        <v>15.89356319143108</v>
       </c>
       <c r="L92" s="131" t="n">
         <v>0</v>
@@ -6757,7 +6757,7 @@
         <v>168.6890429822031</v>
       </c>
       <c r="P92" s="130" t="n">
-        <v>137.9660640772048</v>
+        <v>137.9660640772047</v>
       </c>
       <c r="Q92" s="131" t="n">
         <v>12.14013438652261</v>
@@ -6772,7 +6772,7 @@
         <v>158.2054900284876</v>
       </c>
       <c r="V92" s="130" t="n">
-        <v>129.0017416528368</v>
+        <v>129.0017416528367</v>
       </c>
       <c r="W92" s="131" t="n">
         <v>8.002227321906959</v>
@@ -6876,37 +6876,37 @@
         <v>4251</v>
       </c>
       <c r="J94" s="130" t="n">
-        <v>2701.444887727223</v>
+        <v>2701.444887727222</v>
       </c>
       <c r="K94" s="131" t="n">
         <v>1013.803297948539</v>
       </c>
       <c r="L94" s="131" t="n">
-        <v>264.3214736883766</v>
+        <v>264.3214736883765</v>
       </c>
       <c r="M94" s="131" t="n">
         <v>0</v>
       </c>
       <c r="N94" s="132" t="n">
-        <v>3979.569659364138</v>
+        <v>3979.569659364137</v>
       </c>
       <c r="P94" s="130" t="n">
         <v>2624.318142957748</v>
       </c>
       <c r="Q94" s="131" t="n">
-        <v>978.1421914832282</v>
+        <v>978.1421914832283</v>
       </c>
       <c r="R94" s="131" t="n">
-        <v>255.986103344064</v>
+        <v>255.9861033440639</v>
       </c>
       <c r="S94" s="131" t="n">
         <v>0</v>
       </c>
       <c r="T94" s="132" t="n">
-        <v>3858.44643778504</v>
+        <v>3858.446437785041</v>
       </c>
       <c r="V94" s="130" t="n">
-        <v>2540.109190153185</v>
+        <v>2540.109190153186</v>
       </c>
       <c r="W94" s="131" t="n">
         <v>939.3625222898572</v>
@@ -6918,7 +6918,7 @@
         <v>0</v>
       </c>
       <c r="Z94" s="132" t="n">
-        <v>3726.003239769976</v>
+        <v>3726.003239769977</v>
       </c>
     </row>
     <row r="95">
@@ -7150,7 +7150,7 @@
         <v>32.36265349002131</v>
       </c>
       <c r="L98" s="131" t="n">
-        <v>5.262228230812023</v>
+        <v>5.262228230812022</v>
       </c>
       <c r="M98" s="131" t="n">
         <v>0</v>
@@ -7186,7 +7186,7 @@
         <v>0</v>
       </c>
       <c r="Z98" s="132" t="n">
-        <v>86.19003294722576</v>
+        <v>86.19003294722577</v>
       </c>
     </row>
     <row r="99">
@@ -7217,7 +7217,7 @@
         <v>1628.922856379853</v>
       </c>
       <c r="L99" s="131" t="n">
-        <v>579.4673615811294</v>
+        <v>579.4673615811298</v>
       </c>
       <c r="M99" s="131" t="n">
         <v>19682.11874075477</v>
@@ -7226,34 +7226,34 @@
         <v>27361.36201520906</v>
       </c>
       <c r="P99" s="130" t="n">
-        <v>5717.989908079238</v>
+        <v>5717.989908079231</v>
       </c>
       <c r="Q99" s="131" t="n">
         <v>1677.905544971887</v>
       </c>
       <c r="R99" s="131" t="n">
-        <v>603.0641618903837</v>
+        <v>603.0641618903833</v>
       </c>
       <c r="S99" s="131" t="n">
         <v>21592.61987342794</v>
       </c>
       <c r="T99" s="132" t="n">
-        <v>29591.57948836945</v>
+        <v>29591.57948836944</v>
       </c>
       <c r="V99" s="130" t="n">
-        <v>5996.295669644591</v>
+        <v>5996.295669644584</v>
       </c>
       <c r="W99" s="131" t="n">
-        <v>1742.154527729672</v>
+        <v>1742.154527729668</v>
       </c>
       <c r="X99" s="131" t="n">
-        <v>629.6630878851374</v>
+        <v>629.6630878851365</v>
       </c>
       <c r="Y99" s="131" t="n">
         <v>23717.12306039543</v>
       </c>
       <c r="Z99" s="132" t="n">
-        <v>32085.23634565483</v>
+        <v>32085.23634565482</v>
       </c>
     </row>
     <row r="100">
@@ -7550,13 +7550,13 @@
         <v>70932</v>
       </c>
       <c r="J104" s="142" t="n">
-        <v>28907.74755960872</v>
+        <v>28907.74755960871</v>
       </c>
       <c r="K104" s="143" t="n">
         <v>13611.05787861222</v>
       </c>
       <c r="L104" s="143" t="n">
-        <v>3961.879579104034</v>
+        <v>3961.879579104033</v>
       </c>
       <c r="M104" s="143" t="n">
         <v>19690.79668663907</v>
@@ -8625,10 +8625,10 @@
         </is>
       </c>
       <c r="AH25" s="119" t="n">
-        <v>36479108.3909279</v>
+        <v>36479108.39092791</v>
       </c>
       <c r="AI25" s="46" t="n">
-        <v>47681.20374516814</v>
+        <v>47681.20374516815</v>
       </c>
       <c r="AK25" s="120" t="n">
         <v>1</v>
@@ -9529,7 +9529,7 @@
         </is>
       </c>
       <c r="AH37" s="122" t="n">
-        <v>1625494.155551699</v>
+        <v>1625494.1555517</v>
       </c>
       <c r="AI37" s="56" t="n">
         <v>1968.716811057299</v>
@@ -10516,7 +10516,7 @@
         <v>10902.85394682596</v>
       </c>
       <c r="L54" s="131" t="n">
-        <v>3100.939586379484</v>
+        <v>3100.939586379483</v>
       </c>
       <c r="M54" s="131" t="n">
         <v>0</v>
@@ -10525,19 +10525,19 @@
         <v>34480.29792294405</v>
       </c>
       <c r="P54" s="130" t="n">
-        <v>21660.72763903786</v>
+        <v>21660.72763903787</v>
       </c>
       <c r="Q54" s="131" t="n">
         <v>11377.65923837764</v>
       </c>
       <c r="R54" s="131" t="n">
-        <v>3422.487711428825</v>
+        <v>3422.487711428826</v>
       </c>
       <c r="S54" s="131" t="n">
         <v>0</v>
       </c>
       <c r="T54" s="132" t="n">
-        <v>36460.87458884433</v>
+        <v>36460.87458884434</v>
       </c>
       <c r="V54" s="130" t="n">
         <v>23326.03531108902</v>
@@ -10546,13 +10546,13 @@
         <v>12035.45165849652</v>
       </c>
       <c r="X54" s="131" t="n">
-        <v>3876.170523329414</v>
+        <v>3876.170523329415</v>
       </c>
       <c r="Y54" s="131" t="n">
         <v>0</v>
       </c>
       <c r="Z54" s="132" t="n">
-        <v>39237.65749291495</v>
+        <v>39237.65749291496</v>
       </c>
       <c r="AE54" s="121" t="n">
         <v>6</v>
@@ -10809,7 +10809,7 @@
         <v>1650870.480105934</v>
       </c>
       <c r="AH57" s="56" t="n">
-        <v>4932.342742430019</v>
+        <v>4932.34274243002</v>
       </c>
     </row>
     <row r="58">
@@ -10837,10 +10837,10 @@
         <v>2594.410828881019</v>
       </c>
       <c r="K58" s="131" t="n">
-        <v>985.1537316312742</v>
+        <v>985.1537316312744</v>
       </c>
       <c r="L58" s="131" t="n">
-        <v>255.8945333813836</v>
+        <v>255.8945333813835</v>
       </c>
       <c r="M58" s="131" t="n">
         <v>0</v>
@@ -10852,16 +10852,16 @@
         <v>2524.098090035488</v>
       </c>
       <c r="Q58" s="131" t="n">
-        <v>955.4907245728979</v>
+        <v>955.4907245728981</v>
       </c>
       <c r="R58" s="131" t="n">
-        <v>249.3325380336442</v>
+        <v>249.3325380336441</v>
       </c>
       <c r="S58" s="131" t="n">
         <v>0</v>
       </c>
       <c r="T58" s="132" t="n">
-        <v>3728.921352642029</v>
+        <v>3728.92135264203</v>
       </c>
       <c r="V58" s="130" t="n">
         <v>2448.763529811295</v>
@@ -10876,7 +10876,7 @@
         <v>0</v>
       </c>
       <c r="Z58" s="132" t="n">
-        <v>3615.028403056119</v>
+        <v>3615.02840305612</v>
       </c>
       <c r="AE58" s="121" t="n">
         <v>10</v>
@@ -11164,7 +11164,7 @@
         <v>32.36265349002131</v>
       </c>
       <c r="L62" s="131" t="n">
-        <v>5.262228230812023</v>
+        <v>5.262228230812022</v>
       </c>
       <c r="M62" s="131" t="n">
         <v>0</v>
@@ -11200,7 +11200,7 @@
         <v>0</v>
       </c>
       <c r="Z62" s="132" t="n">
-        <v>86.19003294722576</v>
+        <v>86.19003294722577</v>
       </c>
       <c r="AE62" s="121" t="n">
         <v>14</v>
@@ -11242,10 +11242,10 @@
         <v>5470.853056493306</v>
       </c>
       <c r="K63" s="131" t="n">
-        <v>1628.922856379853</v>
+        <v>1628.922856379852</v>
       </c>
       <c r="L63" s="131" t="n">
-        <v>579.4673615811294</v>
+        <v>579.4673615811298</v>
       </c>
       <c r="M63" s="131" t="n">
         <v>17013.70034841627</v>
@@ -11254,34 +11254,34 @@
         <v>24692.94362287056</v>
       </c>
       <c r="P63" s="130" t="n">
-        <v>5717.989908079238</v>
+        <v>5717.989908079231</v>
       </c>
       <c r="Q63" s="131" t="n">
         <v>1677.905544971887</v>
       </c>
       <c r="R63" s="131" t="n">
-        <v>603.0641618903842</v>
+        <v>603.0641618903837</v>
       </c>
       <c r="S63" s="131" t="n">
         <v>18677.29304011533</v>
       </c>
       <c r="T63" s="132" t="n">
-        <v>26676.25265505684</v>
+        <v>26676.25265505683</v>
       </c>
       <c r="V63" s="130" t="n">
-        <v>5996.295669644594</v>
+        <v>5996.295669644587</v>
       </c>
       <c r="W63" s="131" t="n">
-        <v>1742.154527729672</v>
+        <v>1742.154527729668</v>
       </c>
       <c r="X63" s="131" t="n">
-        <v>629.6630878851374</v>
+        <v>629.6630878851365</v>
       </c>
       <c r="Y63" s="131" t="n">
         <v>20543.90331686658</v>
       </c>
       <c r="Z63" s="132" t="n">
-        <v>28912.01660212599</v>
+        <v>28912.01660212598</v>
       </c>
       <c r="AE63" s="121" t="n">
         <v>15</v>
@@ -11541,7 +11541,7 @@
         </is>
       </c>
       <c r="AG66" s="122" t="n">
-        <v>460011.8910178699</v>
+        <v>460011.8910178698</v>
       </c>
       <c r="AH66" s="56" t="n">
         <v>2351.277226042232</v>
@@ -11656,13 +11656,13 @@
         <v>13549.2931883271</v>
       </c>
       <c r="L68" s="143" t="n">
-        <v>3941.563709572809</v>
+        <v>3941.563709572808</v>
       </c>
       <c r="M68" s="143" t="n">
         <v>17013.70034841627</v>
       </c>
       <c r="N68" s="144" t="n">
-        <v>78603.70350424443</v>
+        <v>78603.70350424442</v>
       </c>
       <c r="P68" s="142" t="n">
         <v>29955.58714387762</v>
@@ -11680,7 +11680,7 @@
         <v>84055.34524985497</v>
       </c>
       <c r="V68" s="142" t="n">
-        <v>31822.07038902595</v>
+        <v>31822.07038902594</v>
       </c>
       <c r="W68" s="143" t="n">
         <v>14731.87121800636</v>
@@ -11927,34 +11927,34 @@
         <v>116</v>
       </c>
       <c r="J72" s="130" t="n">
-        <v>60.36280720546834</v>
+        <v>60.36280720546836</v>
       </c>
       <c r="K72" s="131" t="n">
-        <v>17.22156077641948</v>
+        <v>17.22156077641947</v>
       </c>
       <c r="L72" s="131" t="n">
-        <v>11.88892922423182</v>
+        <v>11.88892922423181</v>
       </c>
       <c r="M72" s="131" t="n">
         <v>0</v>
       </c>
       <c r="N72" s="132" t="n">
-        <v>89.47329720611963</v>
+        <v>89.47329720611964</v>
       </c>
       <c r="P72" s="130" t="n">
-        <v>54.7544447970989</v>
+        <v>54.75444479709888</v>
       </c>
       <c r="Q72" s="131" t="n">
         <v>13.17974339598205</v>
       </c>
       <c r="R72" s="131" t="n">
-        <v>9.1285333020486</v>
+        <v>9.128533302048602</v>
       </c>
       <c r="S72" s="131" t="n">
         <v>0</v>
       </c>
       <c r="T72" s="132" t="n">
-        <v>77.06272149512955</v>
+        <v>77.06272149512952</v>
       </c>
       <c r="V72" s="130" t="n">
         <v>48.60500608217873</v>
@@ -11969,7 +11969,7 @@
         <v>0</v>
       </c>
       <c r="Z72" s="132" t="n">
-        <v>63.00658003928496</v>
+        <v>63.00658003928495</v>
       </c>
     </row>
     <row r="73">
@@ -12064,7 +12064,7 @@
         <v>144.1175339064627</v>
       </c>
       <c r="K74" s="131" t="n">
-        <v>15.89356319143109</v>
+        <v>15.89356319143108</v>
       </c>
       <c r="L74" s="131" t="n">
         <v>0</v>
@@ -12076,7 +12076,7 @@
         <v>168.6890429822031</v>
       </c>
       <c r="P74" s="130" t="n">
-        <v>137.9660640772048</v>
+        <v>137.9660640772047</v>
       </c>
       <c r="Q74" s="131" t="n">
         <v>12.14013438652261</v>
@@ -12091,7 +12091,7 @@
         <v>158.2054900284876</v>
       </c>
       <c r="V74" s="130" t="n">
-        <v>129.0017416528368</v>
+        <v>129.0017416528367</v>
       </c>
       <c r="W74" s="131" t="n">
         <v>8.002227321906959</v>
@@ -12201,7 +12201,7 @@
         <v>28.64956631726437</v>
       </c>
       <c r="L76" s="131" t="n">
-        <v>8.426940306992982</v>
+        <v>8.42694030699298</v>
       </c>
       <c r="M76" s="131" t="n">
         <v>0</v>
@@ -12216,7 +12216,7 @@
         <v>22.65146691033027</v>
       </c>
       <c r="R76" s="131" t="n">
-        <v>6.653565310419796</v>
+        <v>6.653565310419798</v>
       </c>
       <c r="S76" s="131" t="n">
         <v>0</v>
@@ -12225,7 +12225,7 @@
         <v>129.5250851430111</v>
       </c>
       <c r="V76" s="130" t="n">
-        <v>91.34566034189018</v>
+        <v>91.34566034189017</v>
       </c>
       <c r="W76" s="131" t="n">
         <v>15.38658979934373</v>
@@ -12530,13 +12530,13 @@
         <v>2397</v>
       </c>
       <c r="J81" s="130" t="n">
-        <v>0</v>
+        <v>-5.684341886080801e-14</v>
       </c>
       <c r="K81" s="131" t="n">
-        <v>-7.105427357601002e-15</v>
+        <v>0</v>
       </c>
       <c r="L81" s="131" t="n">
-        <v>0</v>
+        <v>3.552713678800501e-15</v>
       </c>
       <c r="M81" s="131" t="n">
         <v>2668.418392338495</v>
@@ -12545,22 +12545,22 @@
         <v>2668.418392338495</v>
       </c>
       <c r="P81" s="130" t="n">
-        <v>0</v>
+        <v>5.684341886080801e-14</v>
       </c>
       <c r="Q81" s="131" t="n">
         <v>0</v>
       </c>
       <c r="R81" s="131" t="n">
-        <v>0</v>
+        <v>-1.77635683940025e-15</v>
       </c>
       <c r="S81" s="131" t="n">
-        <v>2915.32683331261</v>
+        <v>2915.326833312611</v>
       </c>
       <c r="T81" s="132" t="n">
-        <v>2915.32683331261</v>
+        <v>2915.326833312611</v>
       </c>
       <c r="V81" s="130" t="n">
-        <v>-5.684341886080801e-14</v>
+        <v>0</v>
       </c>
       <c r="W81" s="131" t="n">
         <v>-7.105427357601002e-15</v>
@@ -12896,7 +12896,7 @@
         <v>2923.426124877371</v>
       </c>
       <c r="T86" s="144" t="n">
-        <v>4942.501101949607</v>
+        <v>4942.501101949608</v>
       </c>
       <c r="V86" s="142" t="n">
         <v>268.9524080769056</v>
@@ -13132,22 +13132,22 @@
         <v>32117</v>
       </c>
       <c r="J90" s="130" t="n">
-        <v>20536.86719694408</v>
+        <v>20536.86719694407</v>
       </c>
       <c r="K90" s="131" t="n">
         <v>10920.07550760238</v>
       </c>
       <c r="L90" s="131" t="n">
-        <v>3112.828515603716</v>
+        <v>3112.828515603715</v>
       </c>
       <c r="M90" s="131" t="n">
         <v>0</v>
       </c>
       <c r="N90" s="132" t="n">
-        <v>34569.77122015017</v>
+        <v>34569.77122015016</v>
       </c>
       <c r="P90" s="130" t="n">
-        <v>21715.48208383496</v>
+        <v>21715.48208383497</v>
       </c>
       <c r="Q90" s="131" t="n">
         <v>11390.83898177362</v>
@@ -13159,22 +13159,22 @@
         <v>0</v>
       </c>
       <c r="T90" s="132" t="n">
-        <v>36537.93731033946</v>
+        <v>36537.93731033947</v>
       </c>
       <c r="V90" s="130" t="n">
         <v>23374.6403171712</v>
       </c>
       <c r="W90" s="131" t="n">
-        <v>12044.16326397683</v>
+        <v>12044.16326397684</v>
       </c>
       <c r="X90" s="131" t="n">
-        <v>3881.860491806206</v>
+        <v>3881.860491806207</v>
       </c>
       <c r="Y90" s="131" t="n">
         <v>0</v>
       </c>
       <c r="Z90" s="132" t="n">
-        <v>39300.66407295423</v>
+        <v>39300.66407295424</v>
       </c>
     </row>
     <row r="91">
@@ -13269,7 +13269,7 @@
         <v>144.1175339064627</v>
       </c>
       <c r="K92" s="131" t="n">
-        <v>15.89356319143109</v>
+        <v>15.89356319143108</v>
       </c>
       <c r="L92" s="131" t="n">
         <v>0</v>
@@ -13281,7 +13281,7 @@
         <v>168.6890429822031</v>
       </c>
       <c r="P92" s="130" t="n">
-        <v>137.9660640772048</v>
+        <v>137.9660640772047</v>
       </c>
       <c r="Q92" s="131" t="n">
         <v>12.14013438652261</v>
@@ -13296,7 +13296,7 @@
         <v>158.2054900284876</v>
       </c>
       <c r="V92" s="130" t="n">
-        <v>129.0017416528368</v>
+        <v>129.0017416528367</v>
       </c>
       <c r="W92" s="131" t="n">
         <v>8.002227321906959</v>
@@ -13400,37 +13400,37 @@
         <v>4251</v>
       </c>
       <c r="J94" s="130" t="n">
-        <v>2701.444887727223</v>
+        <v>2701.444887727222</v>
       </c>
       <c r="K94" s="131" t="n">
         <v>1013.803297948539</v>
       </c>
       <c r="L94" s="131" t="n">
-        <v>264.3214736883766</v>
+        <v>264.3214736883765</v>
       </c>
       <c r="M94" s="131" t="n">
         <v>0</v>
       </c>
       <c r="N94" s="132" t="n">
-        <v>3979.569659364138</v>
+        <v>3979.569659364137</v>
       </c>
       <c r="P94" s="130" t="n">
         <v>2624.318142957748</v>
       </c>
       <c r="Q94" s="131" t="n">
-        <v>978.1421914832282</v>
+        <v>978.1421914832283</v>
       </c>
       <c r="R94" s="131" t="n">
-        <v>255.986103344064</v>
+        <v>255.9861033440639</v>
       </c>
       <c r="S94" s="131" t="n">
         <v>0</v>
       </c>
       <c r="T94" s="132" t="n">
-        <v>3858.44643778504</v>
+        <v>3858.446437785041</v>
       </c>
       <c r="V94" s="130" t="n">
-        <v>2540.109190153185</v>
+        <v>2540.109190153186</v>
       </c>
       <c r="W94" s="131" t="n">
         <v>939.3625222898572</v>
@@ -13442,7 +13442,7 @@
         <v>0</v>
       </c>
       <c r="Z94" s="132" t="n">
-        <v>3726.003239769976</v>
+        <v>3726.003239769977</v>
       </c>
     </row>
     <row r="95">
@@ -13674,7 +13674,7 @@
         <v>32.36265349002131</v>
       </c>
       <c r="L98" s="131" t="n">
-        <v>5.262228230812023</v>
+        <v>5.262228230812022</v>
       </c>
       <c r="M98" s="131" t="n">
         <v>0</v>
@@ -13710,7 +13710,7 @@
         <v>0</v>
       </c>
       <c r="Z98" s="132" t="n">
-        <v>86.19003294722576</v>
+        <v>86.19003294722577</v>
       </c>
     </row>
     <row r="99">
@@ -13741,7 +13741,7 @@
         <v>1628.922856379853</v>
       </c>
       <c r="L99" s="131" t="n">
-        <v>579.4673615811294</v>
+        <v>579.4673615811298</v>
       </c>
       <c r="M99" s="131" t="n">
         <v>19682.11874075477</v>
@@ -13750,34 +13750,34 @@
         <v>27361.36201520906</v>
       </c>
       <c r="P99" s="130" t="n">
-        <v>5717.989908079238</v>
+        <v>5717.989908079231</v>
       </c>
       <c r="Q99" s="131" t="n">
         <v>1677.905544971887</v>
       </c>
       <c r="R99" s="131" t="n">
-        <v>603.0641618903837</v>
+        <v>603.0641618903833</v>
       </c>
       <c r="S99" s="131" t="n">
         <v>21592.61987342794</v>
       </c>
       <c r="T99" s="132" t="n">
-        <v>29591.57948836945</v>
+        <v>29591.57948836944</v>
       </c>
       <c r="V99" s="130" t="n">
-        <v>5996.295669644591</v>
+        <v>5996.295669644584</v>
       </c>
       <c r="W99" s="131" t="n">
-        <v>1742.154527729672</v>
+        <v>1742.154527729668</v>
       </c>
       <c r="X99" s="131" t="n">
-        <v>629.6630878851374</v>
+        <v>629.6630878851365</v>
       </c>
       <c r="Y99" s="131" t="n">
         <v>23717.12306039543</v>
       </c>
       <c r="Z99" s="132" t="n">
-        <v>32085.23634565483</v>
+        <v>32085.23634565482</v>
       </c>
     </row>
     <row r="100">
@@ -14074,13 +14074,13 @@
         <v>70932</v>
       </c>
       <c r="J104" s="142" t="n">
-        <v>28907.74755960872</v>
+        <v>28907.74755960871</v>
       </c>
       <c r="K104" s="143" t="n">
         <v>13611.05787861222</v>
       </c>
       <c r="L104" s="143" t="n">
-        <v>3961.879579104034</v>
+        <v>3961.879579104033</v>
       </c>
       <c r="M104" s="143" t="n">
         <v>19690.79668663907</v>
@@ -16053,7 +16053,7 @@
         </is>
       </c>
       <c r="AH37" s="122" t="n">
-        <v>1738156.81227514</v>
+        <v>1738156.812275141</v>
       </c>
       <c r="AI37" s="56" t="n">
         <v>2131.779535882219</v>
@@ -16414,10 +16414,10 @@
         </is>
       </c>
       <c r="AH42" s="122" t="n">
-        <v>1241054.16594568</v>
+        <v>1241054.165945679</v>
       </c>
       <c r="AI42" s="56" t="n">
-        <v>82.18910757100559</v>
+        <v>82.18910757100561</v>
       </c>
       <c r="AK42" s="123" t="n">
         <v>18</v>
@@ -17006,7 +17006,7 @@
         </is>
       </c>
       <c r="AG53" s="122" t="n">
-        <v>7773940.370779474</v>
+        <v>7773940.370779475</v>
       </c>
       <c r="AH53" s="56" t="n">
         <v>1037.902475161102</v>
@@ -17040,7 +17040,7 @@
         <v>10902.85394682596</v>
       </c>
       <c r="L54" s="131" t="n">
-        <v>3100.939586379484</v>
+        <v>3100.939586379483</v>
       </c>
       <c r="M54" s="131" t="n">
         <v>0</v>
@@ -17049,19 +17049,19 @@
         <v>34480.29792294405</v>
       </c>
       <c r="P54" s="130" t="n">
-        <v>21660.72763903786</v>
+        <v>21660.72763903787</v>
       </c>
       <c r="Q54" s="131" t="n">
         <v>11377.65923837764</v>
       </c>
       <c r="R54" s="131" t="n">
-        <v>3422.487711428825</v>
+        <v>3422.487711428826</v>
       </c>
       <c r="S54" s="131" t="n">
         <v>0</v>
       </c>
       <c r="T54" s="132" t="n">
-        <v>36460.87458884433</v>
+        <v>36460.87458884434</v>
       </c>
       <c r="V54" s="130" t="n">
         <v>23326.03531108902</v>
@@ -17070,13 +17070,13 @@
         <v>12035.45165849652</v>
       </c>
       <c r="X54" s="131" t="n">
-        <v>3876.170523329414</v>
+        <v>3876.170523329415</v>
       </c>
       <c r="Y54" s="131" t="n">
         <v>0</v>
       </c>
       <c r="Z54" s="132" t="n">
-        <v>39237.65749291495</v>
+        <v>39237.65749291496</v>
       </c>
       <c r="AE54" s="121" t="n">
         <v>6</v>
@@ -17361,10 +17361,10 @@
         <v>2594.410828881019</v>
       </c>
       <c r="K58" s="131" t="n">
-        <v>985.1537316312742</v>
+        <v>985.1537316312744</v>
       </c>
       <c r="L58" s="131" t="n">
-        <v>255.8945333813836</v>
+        <v>255.8945333813835</v>
       </c>
       <c r="M58" s="131" t="n">
         <v>0</v>
@@ -17376,16 +17376,16 @@
         <v>2524.098090035488</v>
       </c>
       <c r="Q58" s="131" t="n">
-        <v>955.4907245728979</v>
+        <v>955.4907245728981</v>
       </c>
       <c r="R58" s="131" t="n">
-        <v>249.3325380336442</v>
+        <v>249.3325380336441</v>
       </c>
       <c r="S58" s="131" t="n">
         <v>0</v>
       </c>
       <c r="T58" s="132" t="n">
-        <v>3728.921352642029</v>
+        <v>3728.92135264203</v>
       </c>
       <c r="V58" s="130" t="n">
         <v>2448.763529811295</v>
@@ -17400,7 +17400,7 @@
         <v>0</v>
       </c>
       <c r="Z58" s="132" t="n">
-        <v>3615.028403056119</v>
+        <v>3615.02840305612</v>
       </c>
       <c r="AE58" s="121" t="n">
         <v>10</v>
@@ -17414,7 +17414,7 @@
         <v>1659794.377793473</v>
       </c>
       <c r="AH58" s="56" t="n">
-        <v>4707.822500794604</v>
+        <v>4707.822500794605</v>
       </c>
     </row>
     <row r="59">
@@ -17688,7 +17688,7 @@
         <v>32.36265349002131</v>
       </c>
       <c r="L62" s="131" t="n">
-        <v>5.262228230812023</v>
+        <v>5.262228230812022</v>
       </c>
       <c r="M62" s="131" t="n">
         <v>0</v>
@@ -17724,7 +17724,7 @@
         <v>0</v>
       </c>
       <c r="Z62" s="132" t="n">
-        <v>86.19003294722576</v>
+        <v>86.19003294722577</v>
       </c>
       <c r="AE62" s="121" t="n">
         <v>14</v>
@@ -17766,10 +17766,10 @@
         <v>5470.853056493306</v>
       </c>
       <c r="K63" s="131" t="n">
-        <v>1628.922856379853</v>
+        <v>1628.922856379852</v>
       </c>
       <c r="L63" s="131" t="n">
-        <v>579.4673615811294</v>
+        <v>579.4673615811298</v>
       </c>
       <c r="M63" s="131" t="n">
         <v>17013.70034841627</v>
@@ -17778,34 +17778,34 @@
         <v>24692.94362287056</v>
       </c>
       <c r="P63" s="130" t="n">
-        <v>5717.989908079238</v>
+        <v>5717.989908079231</v>
       </c>
       <c r="Q63" s="131" t="n">
         <v>1677.905544971887</v>
       </c>
       <c r="R63" s="131" t="n">
-        <v>603.0641618903842</v>
+        <v>603.0641618903837</v>
       </c>
       <c r="S63" s="131" t="n">
         <v>18677.29304011533</v>
       </c>
       <c r="T63" s="132" t="n">
-        <v>26676.25265505684</v>
+        <v>26676.25265505683</v>
       </c>
       <c r="V63" s="130" t="n">
-        <v>5996.295669644594</v>
+        <v>5996.295669644587</v>
       </c>
       <c r="W63" s="131" t="n">
-        <v>1742.154527729672</v>
+        <v>1742.154527729668</v>
       </c>
       <c r="X63" s="131" t="n">
-        <v>629.6630878851374</v>
+        <v>629.6630878851365</v>
       </c>
       <c r="Y63" s="131" t="n">
         <v>20543.90331686658</v>
       </c>
       <c r="Z63" s="132" t="n">
-        <v>28912.01660212599</v>
+        <v>28912.01660212598</v>
       </c>
       <c r="AE63" s="121" t="n">
         <v>15</v>
@@ -18146,7 +18146,7 @@
         </is>
       </c>
       <c r="AG67" s="122" t="n">
-        <v>439850.7482322499</v>
+        <v>439850.74823225</v>
       </c>
       <c r="AH67" s="56" t="n">
         <v>1540.734713659512</v>
@@ -18180,13 +18180,13 @@
         <v>13549.2931883271</v>
       </c>
       <c r="L68" s="143" t="n">
-        <v>3941.563709572809</v>
+        <v>3941.563709572808</v>
       </c>
       <c r="M68" s="143" t="n">
         <v>17013.70034841627</v>
       </c>
       <c r="N68" s="144" t="n">
-        <v>78603.70350424443</v>
+        <v>78603.70350424442</v>
       </c>
       <c r="P68" s="142" t="n">
         <v>29955.58714387762</v>
@@ -18204,7 +18204,7 @@
         <v>84055.34524985497</v>
       </c>
       <c r="V68" s="142" t="n">
-        <v>31822.07038902595</v>
+        <v>31822.07038902594</v>
       </c>
       <c r="W68" s="143" t="n">
         <v>14731.87121800636</v>
@@ -18451,34 +18451,34 @@
         <v>116</v>
       </c>
       <c r="J72" s="130" t="n">
-        <v>60.36280720546834</v>
+        <v>60.36280720546836</v>
       </c>
       <c r="K72" s="131" t="n">
-        <v>17.22156077641948</v>
+        <v>17.22156077641947</v>
       </c>
       <c r="L72" s="131" t="n">
-        <v>11.88892922423182</v>
+        <v>11.88892922423181</v>
       </c>
       <c r="M72" s="131" t="n">
         <v>0</v>
       </c>
       <c r="N72" s="132" t="n">
-        <v>89.47329720611963</v>
+        <v>89.47329720611964</v>
       </c>
       <c r="P72" s="130" t="n">
-        <v>54.7544447970989</v>
+        <v>54.75444479709888</v>
       </c>
       <c r="Q72" s="131" t="n">
         <v>13.17974339598205</v>
       </c>
       <c r="R72" s="131" t="n">
-        <v>9.1285333020486</v>
+        <v>9.128533302048602</v>
       </c>
       <c r="S72" s="131" t="n">
         <v>0</v>
       </c>
       <c r="T72" s="132" t="n">
-        <v>77.06272149512955</v>
+        <v>77.06272149512952</v>
       </c>
       <c r="V72" s="130" t="n">
         <v>48.60500608217873</v>
@@ -18493,7 +18493,7 @@
         <v>0</v>
       </c>
       <c r="Z72" s="132" t="n">
-        <v>63.00658003928496</v>
+        <v>63.00658003928495</v>
       </c>
     </row>
     <row r="73">
@@ -18588,7 +18588,7 @@
         <v>144.1175339064627</v>
       </c>
       <c r="K74" s="131" t="n">
-        <v>15.89356319143109</v>
+        <v>15.89356319143108</v>
       </c>
       <c r="L74" s="131" t="n">
         <v>0</v>
@@ -18600,7 +18600,7 @@
         <v>168.6890429822031</v>
       </c>
       <c r="P74" s="130" t="n">
-        <v>137.9660640772048</v>
+        <v>137.9660640772047</v>
       </c>
       <c r="Q74" s="131" t="n">
         <v>12.14013438652261</v>
@@ -18615,7 +18615,7 @@
         <v>158.2054900284876</v>
       </c>
       <c r="V74" s="130" t="n">
-        <v>129.0017416528368</v>
+        <v>129.0017416528367</v>
       </c>
       <c r="W74" s="131" t="n">
         <v>8.002227321906959</v>
@@ -18725,7 +18725,7 @@
         <v>28.64956631726437</v>
       </c>
       <c r="L76" s="131" t="n">
-        <v>8.426940306992982</v>
+        <v>8.42694030699298</v>
       </c>
       <c r="M76" s="131" t="n">
         <v>0</v>
@@ -18740,7 +18740,7 @@
         <v>22.65146691033027</v>
       </c>
       <c r="R76" s="131" t="n">
-        <v>6.653565310419796</v>
+        <v>6.653565310419798</v>
       </c>
       <c r="S76" s="131" t="n">
         <v>0</v>
@@ -18749,7 +18749,7 @@
         <v>129.5250851430111</v>
       </c>
       <c r="V76" s="130" t="n">
-        <v>91.34566034189018</v>
+        <v>91.34566034189017</v>
       </c>
       <c r="W76" s="131" t="n">
         <v>15.38658979934373</v>
@@ -19054,13 +19054,13 @@
         <v>2397</v>
       </c>
       <c r="J81" s="130" t="n">
-        <v>0</v>
+        <v>-5.684341886080801e-14</v>
       </c>
       <c r="K81" s="131" t="n">
-        <v>-7.105427357601002e-15</v>
+        <v>0</v>
       </c>
       <c r="L81" s="131" t="n">
-        <v>0</v>
+        <v>3.552713678800501e-15</v>
       </c>
       <c r="M81" s="131" t="n">
         <v>2668.418392338495</v>
@@ -19069,22 +19069,22 @@
         <v>2668.418392338495</v>
       </c>
       <c r="P81" s="130" t="n">
-        <v>0</v>
+        <v>5.684341886080801e-14</v>
       </c>
       <c r="Q81" s="131" t="n">
         <v>0</v>
       </c>
       <c r="R81" s="131" t="n">
-        <v>0</v>
+        <v>-1.77635683940025e-15</v>
       </c>
       <c r="S81" s="131" t="n">
-        <v>2915.32683331261</v>
+        <v>2915.326833312611</v>
       </c>
       <c r="T81" s="132" t="n">
-        <v>2915.32683331261</v>
+        <v>2915.326833312611</v>
       </c>
       <c r="V81" s="130" t="n">
-        <v>-5.684341886080801e-14</v>
+        <v>0</v>
       </c>
       <c r="W81" s="131" t="n">
         <v>-7.105427357601002e-15</v>
@@ -19420,7 +19420,7 @@
         <v>2923.426124877371</v>
       </c>
       <c r="T86" s="144" t="n">
-        <v>4942.501101949607</v>
+        <v>4942.501101949608</v>
       </c>
       <c r="V86" s="142" t="n">
         <v>268.9524080769056</v>
@@ -19656,22 +19656,22 @@
         <v>32117</v>
       </c>
       <c r="J90" s="130" t="n">
-        <v>20536.86719694408</v>
+        <v>20536.86719694407</v>
       </c>
       <c r="K90" s="131" t="n">
         <v>10920.07550760238</v>
       </c>
       <c r="L90" s="131" t="n">
-        <v>3112.828515603716</v>
+        <v>3112.828515603715</v>
       </c>
       <c r="M90" s="131" t="n">
         <v>0</v>
       </c>
       <c r="N90" s="132" t="n">
-        <v>34569.77122015017</v>
+        <v>34569.77122015016</v>
       </c>
       <c r="P90" s="130" t="n">
-        <v>21715.48208383496</v>
+        <v>21715.48208383497</v>
       </c>
       <c r="Q90" s="131" t="n">
         <v>11390.83898177362</v>
@@ -19683,22 +19683,22 @@
         <v>0</v>
       </c>
       <c r="T90" s="132" t="n">
-        <v>36537.93731033946</v>
+        <v>36537.93731033947</v>
       </c>
       <c r="V90" s="130" t="n">
         <v>23374.6403171712</v>
       </c>
       <c r="W90" s="131" t="n">
-        <v>12044.16326397683</v>
+        <v>12044.16326397684</v>
       </c>
       <c r="X90" s="131" t="n">
-        <v>3881.860491806206</v>
+        <v>3881.860491806207</v>
       </c>
       <c r="Y90" s="131" t="n">
         <v>0</v>
       </c>
       <c r="Z90" s="132" t="n">
-        <v>39300.66407295423</v>
+        <v>39300.66407295424</v>
       </c>
     </row>
     <row r="91">
@@ -19793,7 +19793,7 @@
         <v>144.1175339064627</v>
       </c>
       <c r="K92" s="131" t="n">
-        <v>15.89356319143109</v>
+        <v>15.89356319143108</v>
       </c>
       <c r="L92" s="131" t="n">
         <v>0</v>
@@ -19805,7 +19805,7 @@
         <v>168.6890429822031</v>
       </c>
       <c r="P92" s="130" t="n">
-        <v>137.9660640772048</v>
+        <v>137.9660640772047</v>
       </c>
       <c r="Q92" s="131" t="n">
         <v>12.14013438652261</v>
@@ -19820,7 +19820,7 @@
         <v>158.2054900284876</v>
       </c>
       <c r="V92" s="130" t="n">
-        <v>129.0017416528368</v>
+        <v>129.0017416528367</v>
       </c>
       <c r="W92" s="131" t="n">
         <v>8.002227321906959</v>
@@ -19924,37 +19924,37 @@
         <v>4251</v>
       </c>
       <c r="J94" s="130" t="n">
-        <v>2701.444887727223</v>
+        <v>2701.444887727222</v>
       </c>
       <c r="K94" s="131" t="n">
         <v>1013.803297948539</v>
       </c>
       <c r="L94" s="131" t="n">
-        <v>264.3214736883766</v>
+        <v>264.3214736883765</v>
       </c>
       <c r="M94" s="131" t="n">
         <v>0</v>
       </c>
       <c r="N94" s="132" t="n">
-        <v>3979.569659364138</v>
+        <v>3979.569659364137</v>
       </c>
       <c r="P94" s="130" t="n">
         <v>2624.318142957748</v>
       </c>
       <c r="Q94" s="131" t="n">
-        <v>978.1421914832282</v>
+        <v>978.1421914832283</v>
       </c>
       <c r="R94" s="131" t="n">
-        <v>255.986103344064</v>
+        <v>255.9861033440639</v>
       </c>
       <c r="S94" s="131" t="n">
         <v>0</v>
       </c>
       <c r="T94" s="132" t="n">
-        <v>3858.44643778504</v>
+        <v>3858.446437785041</v>
       </c>
       <c r="V94" s="130" t="n">
-        <v>2540.109190153185</v>
+        <v>2540.109190153186</v>
       </c>
       <c r="W94" s="131" t="n">
         <v>939.3625222898572</v>
@@ -19966,7 +19966,7 @@
         <v>0</v>
       </c>
       <c r="Z94" s="132" t="n">
-        <v>3726.003239769976</v>
+        <v>3726.003239769977</v>
       </c>
     </row>
     <row r="95">
@@ -20198,7 +20198,7 @@
         <v>32.36265349002131</v>
       </c>
       <c r="L98" s="131" t="n">
-        <v>5.262228230812023</v>
+        <v>5.262228230812022</v>
       </c>
       <c r="M98" s="131" t="n">
         <v>0</v>
@@ -20234,7 +20234,7 @@
         <v>0</v>
       </c>
       <c r="Z98" s="132" t="n">
-        <v>86.19003294722576</v>
+        <v>86.19003294722577</v>
       </c>
     </row>
     <row r="99">
@@ -20265,7 +20265,7 @@
         <v>1628.922856379853</v>
       </c>
       <c r="L99" s="131" t="n">
-        <v>579.4673615811294</v>
+        <v>579.4673615811298</v>
       </c>
       <c r="M99" s="131" t="n">
         <v>19682.11874075477</v>
@@ -20274,34 +20274,34 @@
         <v>27361.36201520906</v>
       </c>
       <c r="P99" s="130" t="n">
-        <v>5717.989908079238</v>
+        <v>5717.989908079231</v>
       </c>
       <c r="Q99" s="131" t="n">
         <v>1677.905544971887</v>
       </c>
       <c r="R99" s="131" t="n">
-        <v>603.0641618903837</v>
+        <v>603.0641618903833</v>
       </c>
       <c r="S99" s="131" t="n">
         <v>21592.61987342794</v>
       </c>
       <c r="T99" s="132" t="n">
-        <v>29591.57948836945</v>
+        <v>29591.57948836944</v>
       </c>
       <c r="V99" s="130" t="n">
-        <v>5996.295669644591</v>
+        <v>5996.295669644584</v>
       </c>
       <c r="W99" s="131" t="n">
-        <v>1742.154527729672</v>
+        <v>1742.154527729668</v>
       </c>
       <c r="X99" s="131" t="n">
-        <v>629.6630878851374</v>
+        <v>629.6630878851365</v>
       </c>
       <c r="Y99" s="131" t="n">
         <v>23717.12306039543</v>
       </c>
       <c r="Z99" s="132" t="n">
-        <v>32085.23634565483</v>
+        <v>32085.23634565482</v>
       </c>
     </row>
     <row r="100">
@@ -20598,13 +20598,13 @@
         <v>70932</v>
       </c>
       <c r="J104" s="142" t="n">
-        <v>28907.74755960872</v>
+        <v>28907.74755960871</v>
       </c>
       <c r="K104" s="143" t="n">
         <v>13611.05787861222</v>
       </c>
       <c r="L104" s="143" t="n">
-        <v>3961.879579104034</v>
+        <v>3961.879579104033</v>
       </c>
       <c r="M104" s="143" t="n">
         <v>19690.79668663907</v>
@@ -21673,10 +21673,10 @@
         </is>
       </c>
       <c r="AH25" s="119" t="n">
-        <v>55719460.42474837</v>
+        <v>55719460.42474838</v>
       </c>
       <c r="AI25" s="46" t="n">
-        <v>68660.92484379245</v>
+        <v>68660.92484379247</v>
       </c>
       <c r="AK25" s="120" t="n">
         <v>1</v>
@@ -22580,7 +22580,7 @@
         <v>2029241.191294712</v>
       </c>
       <c r="AI37" s="56" t="n">
-        <v>3570.123843302601</v>
+        <v>3570.123843302602</v>
       </c>
       <c r="AK37" s="123" t="n">
         <v>13</v>
@@ -22657,7 +22657,7 @@
         <v>1963455.430630518</v>
       </c>
       <c r="AI38" s="56" t="n">
-        <v>2764.956425043126</v>
+        <v>2764.956425043127</v>
       </c>
       <c r="AK38" s="123" t="n">
         <v>14</v>
@@ -23564,7 +23564,7 @@
         <v>10902.85394682596</v>
       </c>
       <c r="L54" s="131" t="n">
-        <v>3100.939586379484</v>
+        <v>3100.939586379483</v>
       </c>
       <c r="M54" s="131" t="n">
         <v>0</v>
@@ -23573,19 +23573,19 @@
         <v>34480.29792294405</v>
       </c>
       <c r="P54" s="130" t="n">
-        <v>21660.72763903786</v>
+        <v>21660.72763903787</v>
       </c>
       <c r="Q54" s="131" t="n">
         <v>11377.65923837764</v>
       </c>
       <c r="R54" s="131" t="n">
-        <v>3422.487711428825</v>
+        <v>3422.487711428826</v>
       </c>
       <c r="S54" s="131" t="n">
         <v>0</v>
       </c>
       <c r="T54" s="132" t="n">
-        <v>36460.87458884433</v>
+        <v>36460.87458884434</v>
       </c>
       <c r="V54" s="130" t="n">
         <v>23326.03531108902</v>
@@ -23594,13 +23594,13 @@
         <v>12035.45165849652</v>
       </c>
       <c r="X54" s="131" t="n">
-        <v>3876.170523329414</v>
+        <v>3876.170523329415</v>
       </c>
       <c r="Y54" s="131" t="n">
         <v>0</v>
       </c>
       <c r="Z54" s="132" t="n">
-        <v>39237.65749291495</v>
+        <v>39237.65749291496</v>
       </c>
       <c r="AE54" s="121" t="n">
         <v>6</v>
@@ -23885,10 +23885,10 @@
         <v>2594.410828881019</v>
       </c>
       <c r="K58" s="131" t="n">
-        <v>985.1537316312742</v>
+        <v>985.1537316312744</v>
       </c>
       <c r="L58" s="131" t="n">
-        <v>255.8945333813836</v>
+        <v>255.8945333813835</v>
       </c>
       <c r="M58" s="131" t="n">
         <v>0</v>
@@ -23900,16 +23900,16 @@
         <v>2524.098090035488</v>
       </c>
       <c r="Q58" s="131" t="n">
-        <v>955.4907245728979</v>
+        <v>955.4907245728981</v>
       </c>
       <c r="R58" s="131" t="n">
-        <v>249.3325380336442</v>
+        <v>249.3325380336441</v>
       </c>
       <c r="S58" s="131" t="n">
         <v>0</v>
       </c>
       <c r="T58" s="132" t="n">
-        <v>3728.921352642029</v>
+        <v>3728.92135264203</v>
       </c>
       <c r="V58" s="130" t="n">
         <v>2448.763529811295</v>
@@ -23924,7 +23924,7 @@
         <v>0</v>
       </c>
       <c r="Z58" s="132" t="n">
-        <v>3615.028403056119</v>
+        <v>3615.02840305612</v>
       </c>
       <c r="AE58" s="121" t="n">
         <v>10</v>
@@ -24181,7 +24181,7 @@
         <v>906466.490944769</v>
       </c>
       <c r="AH61" s="56" t="n">
-        <v>542.4553145801295</v>
+        <v>542.4553145801294</v>
       </c>
     </row>
     <row r="62">
@@ -24212,7 +24212,7 @@
         <v>32.36265349002131</v>
       </c>
       <c r="L62" s="131" t="n">
-        <v>5.262228230812023</v>
+        <v>5.262228230812022</v>
       </c>
       <c r="M62" s="131" t="n">
         <v>0</v>
@@ -24248,7 +24248,7 @@
         <v>0</v>
       </c>
       <c r="Z62" s="132" t="n">
-        <v>86.19003294722576</v>
+        <v>86.19003294722577</v>
       </c>
       <c r="AE62" s="121" t="n">
         <v>14</v>
@@ -24290,10 +24290,10 @@
         <v>5470.853056493306</v>
       </c>
       <c r="K63" s="131" t="n">
-        <v>1628.922856379853</v>
+        <v>1628.922856379852</v>
       </c>
       <c r="L63" s="131" t="n">
-        <v>579.4673615811294</v>
+        <v>579.4673615811298</v>
       </c>
       <c r="M63" s="131" t="n">
         <v>17013.70034841627</v>
@@ -24302,34 +24302,34 @@
         <v>24692.94362287056</v>
       </c>
       <c r="P63" s="130" t="n">
-        <v>5717.989908079238</v>
+        <v>5717.989908079231</v>
       </c>
       <c r="Q63" s="131" t="n">
         <v>1677.905544971887</v>
       </c>
       <c r="R63" s="131" t="n">
-        <v>603.0641618903842</v>
+        <v>603.0641618903837</v>
       </c>
       <c r="S63" s="131" t="n">
         <v>18677.29304011533</v>
       </c>
       <c r="T63" s="132" t="n">
-        <v>26676.25265505684</v>
+        <v>26676.25265505683</v>
       </c>
       <c r="V63" s="130" t="n">
-        <v>5996.295669644594</v>
+        <v>5996.295669644587</v>
       </c>
       <c r="W63" s="131" t="n">
-        <v>1742.154527729672</v>
+        <v>1742.154527729668</v>
       </c>
       <c r="X63" s="131" t="n">
-        <v>629.6630878851374</v>
+        <v>629.6630878851365</v>
       </c>
       <c r="Y63" s="131" t="n">
         <v>20543.90331686658</v>
       </c>
       <c r="Z63" s="132" t="n">
-        <v>28912.01660212599</v>
+        <v>28912.01660212598</v>
       </c>
       <c r="AE63" s="121" t="n">
         <v>15</v>
@@ -24510,7 +24510,7 @@
         <v>412584.2450424846</v>
       </c>
       <c r="AH65" s="56" t="n">
-        <v>765.5601426828616</v>
+        <v>765.5601426828617</v>
       </c>
     </row>
     <row r="66">
@@ -24704,13 +24704,13 @@
         <v>13549.2931883271</v>
       </c>
       <c r="L68" s="143" t="n">
-        <v>3941.563709572809</v>
+        <v>3941.563709572808</v>
       </c>
       <c r="M68" s="143" t="n">
         <v>17013.70034841627</v>
       </c>
       <c r="N68" s="144" t="n">
-        <v>78603.70350424443</v>
+        <v>78603.70350424442</v>
       </c>
       <c r="P68" s="142" t="n">
         <v>29955.58714387762</v>
@@ -24728,7 +24728,7 @@
         <v>84055.34524985497</v>
       </c>
       <c r="V68" s="142" t="n">
-        <v>31822.07038902595</v>
+        <v>31822.07038902594</v>
       </c>
       <c r="W68" s="143" t="n">
         <v>14731.87121800636</v>
@@ -24975,34 +24975,34 @@
         <v>116</v>
       </c>
       <c r="J72" s="130" t="n">
-        <v>60.36280720546834</v>
+        <v>60.36280720546836</v>
       </c>
       <c r="K72" s="131" t="n">
-        <v>17.22156077641948</v>
+        <v>17.22156077641947</v>
       </c>
       <c r="L72" s="131" t="n">
-        <v>11.88892922423182</v>
+        <v>11.88892922423181</v>
       </c>
       <c r="M72" s="131" t="n">
         <v>0</v>
       </c>
       <c r="N72" s="132" t="n">
-        <v>89.47329720611963</v>
+        <v>89.47329720611964</v>
       </c>
       <c r="P72" s="130" t="n">
-        <v>54.7544447970989</v>
+        <v>54.75444479709888</v>
       </c>
       <c r="Q72" s="131" t="n">
         <v>13.17974339598205</v>
       </c>
       <c r="R72" s="131" t="n">
-        <v>9.1285333020486</v>
+        <v>9.128533302048602</v>
       </c>
       <c r="S72" s="131" t="n">
         <v>0</v>
       </c>
       <c r="T72" s="132" t="n">
-        <v>77.06272149512955</v>
+        <v>77.06272149512952</v>
       </c>
       <c r="V72" s="130" t="n">
         <v>48.60500608217873</v>
@@ -25017,7 +25017,7 @@
         <v>0</v>
       </c>
       <c r="Z72" s="132" t="n">
-        <v>63.00658003928496</v>
+        <v>63.00658003928495</v>
       </c>
     </row>
     <row r="73">
@@ -25112,7 +25112,7 @@
         <v>144.1175339064627</v>
       </c>
       <c r="K74" s="131" t="n">
-        <v>15.89356319143109</v>
+        <v>15.89356319143108</v>
       </c>
       <c r="L74" s="131" t="n">
         <v>0</v>
@@ -25124,7 +25124,7 @@
         <v>168.6890429822031</v>
       </c>
       <c r="P74" s="130" t="n">
-        <v>137.9660640772048</v>
+        <v>137.9660640772047</v>
       </c>
       <c r="Q74" s="131" t="n">
         <v>12.14013438652261</v>
@@ -25139,7 +25139,7 @@
         <v>158.2054900284876</v>
       </c>
       <c r="V74" s="130" t="n">
-        <v>129.0017416528368</v>
+        <v>129.0017416528367</v>
       </c>
       <c r="W74" s="131" t="n">
         <v>8.002227321906959</v>
@@ -25249,7 +25249,7 @@
         <v>28.64956631726437</v>
       </c>
       <c r="L76" s="131" t="n">
-        <v>8.426940306992982</v>
+        <v>8.42694030699298</v>
       </c>
       <c r="M76" s="131" t="n">
         <v>0</v>
@@ -25264,7 +25264,7 @@
         <v>22.65146691033027</v>
       </c>
       <c r="R76" s="131" t="n">
-        <v>6.653565310419796</v>
+        <v>6.653565310419798</v>
       </c>
       <c r="S76" s="131" t="n">
         <v>0</v>
@@ -25273,7 +25273,7 @@
         <v>129.5250851430111</v>
       </c>
       <c r="V76" s="130" t="n">
-        <v>91.34566034189018</v>
+        <v>91.34566034189017</v>
       </c>
       <c r="W76" s="131" t="n">
         <v>15.38658979934373</v>
@@ -25578,13 +25578,13 @@
         <v>2397</v>
       </c>
       <c r="J81" s="130" t="n">
-        <v>0</v>
+        <v>-5.684341886080801e-14</v>
       </c>
       <c r="K81" s="131" t="n">
-        <v>-7.105427357601002e-15</v>
+        <v>0</v>
       </c>
       <c r="L81" s="131" t="n">
-        <v>0</v>
+        <v>3.552713678800501e-15</v>
       </c>
       <c r="M81" s="131" t="n">
         <v>2668.418392338495</v>
@@ -25593,22 +25593,22 @@
         <v>2668.418392338495</v>
       </c>
       <c r="P81" s="130" t="n">
-        <v>0</v>
+        <v>5.684341886080801e-14</v>
       </c>
       <c r="Q81" s="131" t="n">
         <v>0</v>
       </c>
       <c r="R81" s="131" t="n">
-        <v>0</v>
+        <v>-1.77635683940025e-15</v>
       </c>
       <c r="S81" s="131" t="n">
-        <v>2915.32683331261</v>
+        <v>2915.326833312611</v>
       </c>
       <c r="T81" s="132" t="n">
-        <v>2915.32683331261</v>
+        <v>2915.326833312611</v>
       </c>
       <c r="V81" s="130" t="n">
-        <v>-5.684341886080801e-14</v>
+        <v>0</v>
       </c>
       <c r="W81" s="131" t="n">
         <v>-7.105427357601002e-15</v>
@@ -25944,7 +25944,7 @@
         <v>2923.426124877371</v>
       </c>
       <c r="T86" s="144" t="n">
-        <v>4942.501101949607</v>
+        <v>4942.501101949608</v>
       </c>
       <c r="V86" s="142" t="n">
         <v>268.9524080769056</v>
@@ -26180,22 +26180,22 @@
         <v>32117</v>
       </c>
       <c r="J90" s="130" t="n">
-        <v>20536.86719694408</v>
+        <v>20536.86719694407</v>
       </c>
       <c r="K90" s="131" t="n">
         <v>10920.07550760238</v>
       </c>
       <c r="L90" s="131" t="n">
-        <v>3112.828515603716</v>
+        <v>3112.828515603715</v>
       </c>
       <c r="M90" s="131" t="n">
         <v>0</v>
       </c>
       <c r="N90" s="132" t="n">
-        <v>34569.77122015017</v>
+        <v>34569.77122015016</v>
       </c>
       <c r="P90" s="130" t="n">
-        <v>21715.48208383496</v>
+        <v>21715.48208383497</v>
       </c>
       <c r="Q90" s="131" t="n">
         <v>11390.83898177362</v>
@@ -26207,22 +26207,22 @@
         <v>0</v>
       </c>
       <c r="T90" s="132" t="n">
-        <v>36537.93731033946</v>
+        <v>36537.93731033947</v>
       </c>
       <c r="V90" s="130" t="n">
         <v>23374.6403171712</v>
       </c>
       <c r="W90" s="131" t="n">
-        <v>12044.16326397683</v>
+        <v>12044.16326397684</v>
       </c>
       <c r="X90" s="131" t="n">
-        <v>3881.860491806206</v>
+        <v>3881.860491806207</v>
       </c>
       <c r="Y90" s="131" t="n">
         <v>0</v>
       </c>
       <c r="Z90" s="132" t="n">
-        <v>39300.66407295423</v>
+        <v>39300.66407295424</v>
       </c>
     </row>
     <row r="91">
@@ -26317,7 +26317,7 @@
         <v>144.1175339064627</v>
       </c>
       <c r="K92" s="131" t="n">
-        <v>15.89356319143109</v>
+        <v>15.89356319143108</v>
       </c>
       <c r="L92" s="131" t="n">
         <v>0</v>
@@ -26329,7 +26329,7 @@
         <v>168.6890429822031</v>
       </c>
       <c r="P92" s="130" t="n">
-        <v>137.9660640772048</v>
+        <v>137.9660640772047</v>
       </c>
       <c r="Q92" s="131" t="n">
         <v>12.14013438652261</v>
@@ -26344,7 +26344,7 @@
         <v>158.2054900284876</v>
       </c>
       <c r="V92" s="130" t="n">
-        <v>129.0017416528368</v>
+        <v>129.0017416528367</v>
       </c>
       <c r="W92" s="131" t="n">
         <v>8.002227321906959</v>
@@ -26448,37 +26448,37 @@
         <v>4251</v>
       </c>
       <c r="J94" s="130" t="n">
-        <v>2701.444887727223</v>
+        <v>2701.444887727222</v>
       </c>
       <c r="K94" s="131" t="n">
         <v>1013.803297948539</v>
       </c>
       <c r="L94" s="131" t="n">
-        <v>264.3214736883766</v>
+        <v>264.3214736883765</v>
       </c>
       <c r="M94" s="131" t="n">
         <v>0</v>
       </c>
       <c r="N94" s="132" t="n">
-        <v>3979.569659364138</v>
+        <v>3979.569659364137</v>
       </c>
       <c r="P94" s="130" t="n">
         <v>2624.318142957748</v>
       </c>
       <c r="Q94" s="131" t="n">
-        <v>978.1421914832282</v>
+        <v>978.1421914832283</v>
       </c>
       <c r="R94" s="131" t="n">
-        <v>255.986103344064</v>
+        <v>255.9861033440639</v>
       </c>
       <c r="S94" s="131" t="n">
         <v>0</v>
       </c>
       <c r="T94" s="132" t="n">
-        <v>3858.44643778504</v>
+        <v>3858.446437785041</v>
       </c>
       <c r="V94" s="130" t="n">
-        <v>2540.109190153185</v>
+        <v>2540.109190153186</v>
       </c>
       <c r="W94" s="131" t="n">
         <v>939.3625222898572</v>
@@ -26490,7 +26490,7 @@
         <v>0</v>
       </c>
       <c r="Z94" s="132" t="n">
-        <v>3726.003239769976</v>
+        <v>3726.003239769977</v>
       </c>
     </row>
     <row r="95">
@@ -26722,7 +26722,7 @@
         <v>32.36265349002131</v>
       </c>
       <c r="L98" s="131" t="n">
-        <v>5.262228230812023</v>
+        <v>5.262228230812022</v>
       </c>
       <c r="M98" s="131" t="n">
         <v>0</v>
@@ -26758,7 +26758,7 @@
         <v>0</v>
       </c>
       <c r="Z98" s="132" t="n">
-        <v>86.19003294722576</v>
+        <v>86.19003294722577</v>
       </c>
     </row>
     <row r="99">
@@ -26789,7 +26789,7 @@
         <v>1628.922856379853</v>
       </c>
       <c r="L99" s="131" t="n">
-        <v>579.4673615811294</v>
+        <v>579.4673615811298</v>
       </c>
       <c r="M99" s="131" t="n">
         <v>19682.11874075477</v>
@@ -26798,34 +26798,34 @@
         <v>27361.36201520906</v>
       </c>
       <c r="P99" s="130" t="n">
-        <v>5717.989908079238</v>
+        <v>5717.989908079231</v>
       </c>
       <c r="Q99" s="131" t="n">
         <v>1677.905544971887</v>
       </c>
       <c r="R99" s="131" t="n">
-        <v>603.0641618903837</v>
+        <v>603.0641618903833</v>
       </c>
       <c r="S99" s="131" t="n">
         <v>21592.61987342794</v>
       </c>
       <c r="T99" s="132" t="n">
-        <v>29591.57948836945</v>
+        <v>29591.57948836944</v>
       </c>
       <c r="V99" s="130" t="n">
-        <v>5996.295669644591</v>
+        <v>5996.295669644584</v>
       </c>
       <c r="W99" s="131" t="n">
-        <v>1742.154527729672</v>
+        <v>1742.154527729668</v>
       </c>
       <c r="X99" s="131" t="n">
-        <v>629.6630878851374</v>
+        <v>629.6630878851365</v>
       </c>
       <c r="Y99" s="131" t="n">
         <v>23717.12306039543</v>
       </c>
       <c r="Z99" s="132" t="n">
-        <v>32085.23634565483</v>
+        <v>32085.23634565482</v>
       </c>
     </row>
     <row r="100">
@@ -27122,13 +27122,13 @@
         <v>70932</v>
       </c>
       <c r="J104" s="142" t="n">
-        <v>28907.74755960872</v>
+        <v>28907.74755960871</v>
       </c>
       <c r="K104" s="143" t="n">
         <v>13611.05787861222</v>
       </c>
       <c r="L104" s="143" t="n">
-        <v>3961.879579104034</v>
+        <v>3961.879579104033</v>
       </c>
       <c r="M104" s="143" t="n">
         <v>19690.79668663907</v>
@@ -28197,10 +28197,10 @@
         </is>
       </c>
       <c r="AH25" s="119" t="n">
-        <v>69285584.18914481</v>
+        <v>69285584.18914482</v>
       </c>
       <c r="AI25" s="46" t="n">
-        <v>82393.10616487112</v>
+        <v>82393.1061648711</v>
       </c>
       <c r="AK25" s="120" t="n">
         <v>1</v>
@@ -28274,7 +28274,7 @@
         </is>
       </c>
       <c r="AH26" s="122" t="n">
-        <v>17597343.42452665</v>
+        <v>17597343.42452664</v>
       </c>
       <c r="AI26" s="56" t="n">
         <v>19791.41132971137</v>
@@ -29244,7 +29244,7 @@
         <v>1704572.018423962</v>
       </c>
       <c r="AI39" s="56" t="n">
-        <v>1964.648020269053</v>
+        <v>1964.648020269052</v>
       </c>
       <c r="AK39" s="123" t="n">
         <v>15</v>
@@ -29311,7 +29311,7 @@
         <v>1628208.049291219</v>
       </c>
       <c r="AI40" s="56" t="n">
-        <v>2218.827294049513</v>
+        <v>2218.827294049512</v>
       </c>
       <c r="AK40" s="123" t="n">
         <v>16</v>
@@ -29462,7 +29462,7 @@
         </is>
       </c>
       <c r="AH42" s="122" t="n">
-        <v>1451451.325188483</v>
+        <v>1451451.325188484</v>
       </c>
       <c r="AI42" s="56" t="n">
         <v>2609.80587903714</v>
@@ -29539,7 +29539,7 @@
         </is>
       </c>
       <c r="AH43" s="122" t="n">
-        <v>1228257.186556878</v>
+        <v>1228257.186556879</v>
       </c>
       <c r="AI43" s="56" t="n">
         <v>1040.245562303857</v>
@@ -30054,7 +30054,7 @@
         </is>
       </c>
       <c r="AG53" s="122" t="n">
-        <v>10455728.23420106</v>
+        <v>10455728.23420105</v>
       </c>
       <c r="AH53" s="56" t="n">
         <v>0</v>
@@ -30088,7 +30088,7 @@
         <v>10902.85394682596</v>
       </c>
       <c r="L54" s="131" t="n">
-        <v>3100.939586379484</v>
+        <v>3100.939586379483</v>
       </c>
       <c r="M54" s="131" t="n">
         <v>0</v>
@@ -30097,19 +30097,19 @@
         <v>34480.29792294405</v>
       </c>
       <c r="P54" s="130" t="n">
-        <v>21660.72763903786</v>
+        <v>21660.72763903787</v>
       </c>
       <c r="Q54" s="131" t="n">
         <v>11377.65923837764</v>
       </c>
       <c r="R54" s="131" t="n">
-        <v>3422.487711428825</v>
+        <v>3422.487711428826</v>
       </c>
       <c r="S54" s="131" t="n">
         <v>0</v>
       </c>
       <c r="T54" s="132" t="n">
-        <v>36460.87458884433</v>
+        <v>36460.87458884434</v>
       </c>
       <c r="V54" s="130" t="n">
         <v>23326.03531108902</v>
@@ -30118,13 +30118,13 @@
         <v>12035.45165849652</v>
       </c>
       <c r="X54" s="131" t="n">
-        <v>3876.170523329414</v>
+        <v>3876.170523329415</v>
       </c>
       <c r="Y54" s="131" t="n">
         <v>0</v>
       </c>
       <c r="Z54" s="132" t="n">
-        <v>39237.65749291495</v>
+        <v>39237.65749291496</v>
       </c>
       <c r="AE54" s="121" t="n">
         <v>6</v>
@@ -30409,10 +30409,10 @@
         <v>2594.410828881019</v>
       </c>
       <c r="K58" s="131" t="n">
-        <v>985.1537316312742</v>
+        <v>985.1537316312744</v>
       </c>
       <c r="L58" s="131" t="n">
-        <v>255.8945333813836</v>
+        <v>255.8945333813835</v>
       </c>
       <c r="M58" s="131" t="n">
         <v>0</v>
@@ -30424,16 +30424,16 @@
         <v>2524.098090035488</v>
       </c>
       <c r="Q58" s="131" t="n">
-        <v>955.4907245728979</v>
+        <v>955.4907245728981</v>
       </c>
       <c r="R58" s="131" t="n">
-        <v>249.3325380336442</v>
+        <v>249.3325380336441</v>
       </c>
       <c r="S58" s="131" t="n">
         <v>0</v>
       </c>
       <c r="T58" s="132" t="n">
-        <v>3728.921352642029</v>
+        <v>3728.92135264203</v>
       </c>
       <c r="V58" s="130" t="n">
         <v>2448.763529811295</v>
@@ -30448,7 +30448,7 @@
         <v>0</v>
       </c>
       <c r="Z58" s="132" t="n">
-        <v>3615.028403056119</v>
+        <v>3615.02840305612</v>
       </c>
       <c r="AE58" s="121" t="n">
         <v>10</v>
@@ -30462,7 +30462,7 @@
         <v>1648512.402877569</v>
       </c>
       <c r="AH58" s="56" t="n">
-        <v>4278.46888204873</v>
+        <v>4278.468882048729</v>
       </c>
     </row>
     <row r="59">
@@ -30540,7 +30540,7 @@
         </is>
       </c>
       <c r="AG59" s="122" t="n">
-        <v>1524240.900547113</v>
+        <v>1524240.900547112</v>
       </c>
       <c r="AH59" s="56" t="n">
         <v>1226.085092929029</v>
@@ -30736,7 +30736,7 @@
         <v>32.36265349002131</v>
       </c>
       <c r="L62" s="131" t="n">
-        <v>5.262228230812023</v>
+        <v>5.262228230812022</v>
       </c>
       <c r="M62" s="131" t="n">
         <v>0</v>
@@ -30772,7 +30772,7 @@
         <v>0</v>
       </c>
       <c r="Z62" s="132" t="n">
-        <v>86.19003294722576</v>
+        <v>86.19003294722577</v>
       </c>
       <c r="AE62" s="121" t="n">
         <v>14</v>
@@ -30814,10 +30814,10 @@
         <v>5470.853056493306</v>
       </c>
       <c r="K63" s="131" t="n">
-        <v>1628.922856379853</v>
+        <v>1628.922856379852</v>
       </c>
       <c r="L63" s="131" t="n">
-        <v>579.4673615811294</v>
+        <v>579.4673615811298</v>
       </c>
       <c r="M63" s="131" t="n">
         <v>17013.70034841627</v>
@@ -30826,34 +30826,34 @@
         <v>24692.94362287056</v>
       </c>
       <c r="P63" s="130" t="n">
-        <v>5717.989908079238</v>
+        <v>5717.989908079231</v>
       </c>
       <c r="Q63" s="131" t="n">
         <v>1677.905544971887</v>
       </c>
       <c r="R63" s="131" t="n">
-        <v>603.0641618903842</v>
+        <v>603.0641618903837</v>
       </c>
       <c r="S63" s="131" t="n">
         <v>18677.29304011533</v>
       </c>
       <c r="T63" s="132" t="n">
-        <v>26676.25265505684</v>
+        <v>26676.25265505683</v>
       </c>
       <c r="V63" s="130" t="n">
-        <v>5996.295669644594</v>
+        <v>5996.295669644587</v>
       </c>
       <c r="W63" s="131" t="n">
-        <v>1742.154527729672</v>
+        <v>1742.154527729668</v>
       </c>
       <c r="X63" s="131" t="n">
-        <v>629.6630878851374</v>
+        <v>629.6630878851365</v>
       </c>
       <c r="Y63" s="131" t="n">
         <v>20543.90331686658</v>
       </c>
       <c r="Z63" s="132" t="n">
-        <v>28912.01660212599</v>
+        <v>28912.01660212598</v>
       </c>
       <c r="AE63" s="121" t="n">
         <v>15</v>
@@ -31228,13 +31228,13 @@
         <v>13549.2931883271</v>
       </c>
       <c r="L68" s="143" t="n">
-        <v>3941.563709572809</v>
+        <v>3941.563709572808</v>
       </c>
       <c r="M68" s="143" t="n">
         <v>17013.70034841627</v>
       </c>
       <c r="N68" s="144" t="n">
-        <v>78603.70350424443</v>
+        <v>78603.70350424442</v>
       </c>
       <c r="P68" s="142" t="n">
         <v>29955.58714387762</v>
@@ -31252,7 +31252,7 @@
         <v>84055.34524985497</v>
       </c>
       <c r="V68" s="142" t="n">
-        <v>31822.07038902595</v>
+        <v>31822.07038902594</v>
       </c>
       <c r="W68" s="143" t="n">
         <v>14731.87121800636</v>
@@ -31499,34 +31499,34 @@
         <v>116</v>
       </c>
       <c r="J72" s="130" t="n">
-        <v>60.36280720546834</v>
+        <v>60.36280720546836</v>
       </c>
       <c r="K72" s="131" t="n">
-        <v>17.22156077641948</v>
+        <v>17.22156077641947</v>
       </c>
       <c r="L72" s="131" t="n">
-        <v>11.88892922423182</v>
+        <v>11.88892922423181</v>
       </c>
       <c r="M72" s="131" t="n">
         <v>0</v>
       </c>
       <c r="N72" s="132" t="n">
-        <v>89.47329720611963</v>
+        <v>89.47329720611964</v>
       </c>
       <c r="P72" s="130" t="n">
-        <v>54.7544447970989</v>
+        <v>54.75444479709888</v>
       </c>
       <c r="Q72" s="131" t="n">
         <v>13.17974339598205</v>
       </c>
       <c r="R72" s="131" t="n">
-        <v>9.1285333020486</v>
+        <v>9.128533302048602</v>
       </c>
       <c r="S72" s="131" t="n">
         <v>0</v>
       </c>
       <c r="T72" s="132" t="n">
-        <v>77.06272149512955</v>
+        <v>77.06272149512952</v>
       </c>
       <c r="V72" s="130" t="n">
         <v>48.60500608217873</v>
@@ -31541,7 +31541,7 @@
         <v>0</v>
       </c>
       <c r="Z72" s="132" t="n">
-        <v>63.00658003928496</v>
+        <v>63.00658003928495</v>
       </c>
     </row>
     <row r="73">
@@ -31636,7 +31636,7 @@
         <v>144.1175339064627</v>
       </c>
       <c r="K74" s="131" t="n">
-        <v>15.89356319143109</v>
+        <v>15.89356319143108</v>
       </c>
       <c r="L74" s="131" t="n">
         <v>0</v>
@@ -31648,7 +31648,7 @@
         <v>168.6890429822031</v>
       </c>
       <c r="P74" s="130" t="n">
-        <v>137.9660640772048</v>
+        <v>137.9660640772047</v>
       </c>
       <c r="Q74" s="131" t="n">
         <v>12.14013438652261</v>
@@ -31663,7 +31663,7 @@
         <v>158.2054900284876</v>
       </c>
       <c r="V74" s="130" t="n">
-        <v>129.0017416528368</v>
+        <v>129.0017416528367</v>
       </c>
       <c r="W74" s="131" t="n">
         <v>8.002227321906959</v>
@@ -31773,7 +31773,7 @@
         <v>28.64956631726437</v>
       </c>
       <c r="L76" s="131" t="n">
-        <v>8.426940306992982</v>
+        <v>8.42694030699298</v>
       </c>
       <c r="M76" s="131" t="n">
         <v>0</v>
@@ -31788,7 +31788,7 @@
         <v>22.65146691033027</v>
       </c>
       <c r="R76" s="131" t="n">
-        <v>6.653565310419796</v>
+        <v>6.653565310419798</v>
       </c>
       <c r="S76" s="131" t="n">
         <v>0</v>
@@ -31797,7 +31797,7 @@
         <v>129.5250851430111</v>
       </c>
       <c r="V76" s="130" t="n">
-        <v>91.34566034189018</v>
+        <v>91.34566034189017</v>
       </c>
       <c r="W76" s="131" t="n">
         <v>15.38658979934373</v>
@@ -32102,13 +32102,13 @@
         <v>2397</v>
       </c>
       <c r="J81" s="130" t="n">
-        <v>0</v>
+        <v>-5.684341886080801e-14</v>
       </c>
       <c r="K81" s="131" t="n">
-        <v>-7.105427357601002e-15</v>
+        <v>0</v>
       </c>
       <c r="L81" s="131" t="n">
-        <v>0</v>
+        <v>3.552713678800501e-15</v>
       </c>
       <c r="M81" s="131" t="n">
         <v>2668.418392338495</v>
@@ -32117,22 +32117,22 @@
         <v>2668.418392338495</v>
       </c>
       <c r="P81" s="130" t="n">
-        <v>0</v>
+        <v>5.684341886080801e-14</v>
       </c>
       <c r="Q81" s="131" t="n">
         <v>0</v>
       </c>
       <c r="R81" s="131" t="n">
-        <v>0</v>
+        <v>-1.77635683940025e-15</v>
       </c>
       <c r="S81" s="131" t="n">
-        <v>2915.32683331261</v>
+        <v>2915.326833312611</v>
       </c>
       <c r="T81" s="132" t="n">
-        <v>2915.32683331261</v>
+        <v>2915.326833312611</v>
       </c>
       <c r="V81" s="130" t="n">
-        <v>-5.684341886080801e-14</v>
+        <v>0</v>
       </c>
       <c r="W81" s="131" t="n">
         <v>-7.105427357601002e-15</v>
@@ -32468,7 +32468,7 @@
         <v>2923.426124877371</v>
       </c>
       <c r="T86" s="144" t="n">
-        <v>4942.501101949607</v>
+        <v>4942.501101949608</v>
       </c>
       <c r="V86" s="142" t="n">
         <v>268.9524080769056</v>
@@ -32704,22 +32704,22 @@
         <v>32117</v>
       </c>
       <c r="J90" s="130" t="n">
-        <v>20536.86719694408</v>
+        <v>20536.86719694407</v>
       </c>
       <c r="K90" s="131" t="n">
         <v>10920.07550760238</v>
       </c>
       <c r="L90" s="131" t="n">
-        <v>3112.828515603716</v>
+        <v>3112.828515603715</v>
       </c>
       <c r="M90" s="131" t="n">
         <v>0</v>
       </c>
       <c r="N90" s="132" t="n">
-        <v>34569.77122015017</v>
+        <v>34569.77122015016</v>
       </c>
       <c r="P90" s="130" t="n">
-        <v>21715.48208383496</v>
+        <v>21715.48208383497</v>
       </c>
       <c r="Q90" s="131" t="n">
         <v>11390.83898177362</v>
@@ -32731,22 +32731,22 @@
         <v>0</v>
       </c>
       <c r="T90" s="132" t="n">
-        <v>36537.93731033946</v>
+        <v>36537.93731033947</v>
       </c>
       <c r="V90" s="130" t="n">
         <v>23374.6403171712</v>
       </c>
       <c r="W90" s="131" t="n">
-        <v>12044.16326397683</v>
+        <v>12044.16326397684</v>
       </c>
       <c r="X90" s="131" t="n">
-        <v>3881.860491806206</v>
+        <v>3881.860491806207</v>
       </c>
       <c r="Y90" s="131" t="n">
         <v>0</v>
       </c>
       <c r="Z90" s="132" t="n">
-        <v>39300.66407295423</v>
+        <v>39300.66407295424</v>
       </c>
     </row>
     <row r="91">
@@ -32841,7 +32841,7 @@
         <v>144.1175339064627</v>
       </c>
       <c r="K92" s="131" t="n">
-        <v>15.89356319143109</v>
+        <v>15.89356319143108</v>
       </c>
       <c r="L92" s="131" t="n">
         <v>0</v>
@@ -32853,7 +32853,7 @@
         <v>168.6890429822031</v>
       </c>
       <c r="P92" s="130" t="n">
-        <v>137.9660640772048</v>
+        <v>137.9660640772047</v>
       </c>
       <c r="Q92" s="131" t="n">
         <v>12.14013438652261</v>
@@ -32868,7 +32868,7 @@
         <v>158.2054900284876</v>
       </c>
       <c r="V92" s="130" t="n">
-        <v>129.0017416528368</v>
+        <v>129.0017416528367</v>
       </c>
       <c r="W92" s="131" t="n">
         <v>8.002227321906959</v>
@@ -32972,37 +32972,37 @@
         <v>4251</v>
       </c>
       <c r="J94" s="130" t="n">
-        <v>2701.444887727223</v>
+        <v>2701.444887727222</v>
       </c>
       <c r="K94" s="131" t="n">
         <v>1013.803297948539</v>
       </c>
       <c r="L94" s="131" t="n">
-        <v>264.3214736883766</v>
+        <v>264.3214736883765</v>
       </c>
       <c r="M94" s="131" t="n">
         <v>0</v>
       </c>
       <c r="N94" s="132" t="n">
-        <v>3979.569659364138</v>
+        <v>3979.569659364137</v>
       </c>
       <c r="P94" s="130" t="n">
         <v>2624.318142957748</v>
       </c>
       <c r="Q94" s="131" t="n">
-        <v>978.1421914832282</v>
+        <v>978.1421914832283</v>
       </c>
       <c r="R94" s="131" t="n">
-        <v>255.986103344064</v>
+        <v>255.9861033440639</v>
       </c>
       <c r="S94" s="131" t="n">
         <v>0</v>
       </c>
       <c r="T94" s="132" t="n">
-        <v>3858.44643778504</v>
+        <v>3858.446437785041</v>
       </c>
       <c r="V94" s="130" t="n">
-        <v>2540.109190153185</v>
+        <v>2540.109190153186</v>
       </c>
       <c r="W94" s="131" t="n">
         <v>939.3625222898572</v>
@@ -33014,7 +33014,7 @@
         <v>0</v>
       </c>
       <c r="Z94" s="132" t="n">
-        <v>3726.003239769976</v>
+        <v>3726.003239769977</v>
       </c>
     </row>
     <row r="95">
@@ -33246,7 +33246,7 @@
         <v>32.36265349002131</v>
       </c>
       <c r="L98" s="131" t="n">
-        <v>5.262228230812023</v>
+        <v>5.262228230812022</v>
       </c>
       <c r="M98" s="131" t="n">
         <v>0</v>
@@ -33282,7 +33282,7 @@
         <v>0</v>
       </c>
       <c r="Z98" s="132" t="n">
-        <v>86.19003294722576</v>
+        <v>86.19003294722577</v>
       </c>
     </row>
     <row r="99">
@@ -33313,7 +33313,7 @@
         <v>1628.922856379853</v>
       </c>
       <c r="L99" s="131" t="n">
-        <v>579.4673615811294</v>
+        <v>579.4673615811298</v>
       </c>
       <c r="M99" s="131" t="n">
         <v>19682.11874075477</v>
@@ -33322,34 +33322,34 @@
         <v>27361.36201520906</v>
       </c>
       <c r="P99" s="130" t="n">
-        <v>5717.989908079238</v>
+        <v>5717.989908079231</v>
       </c>
       <c r="Q99" s="131" t="n">
         <v>1677.905544971887</v>
       </c>
       <c r="R99" s="131" t="n">
-        <v>603.0641618903837</v>
+        <v>603.0641618903833</v>
       </c>
       <c r="S99" s="131" t="n">
         <v>21592.61987342794</v>
       </c>
       <c r="T99" s="132" t="n">
-        <v>29591.57948836945</v>
+        <v>29591.57948836944</v>
       </c>
       <c r="V99" s="130" t="n">
-        <v>5996.295669644591</v>
+        <v>5996.295669644584</v>
       </c>
       <c r="W99" s="131" t="n">
-        <v>1742.154527729672</v>
+        <v>1742.154527729668</v>
       </c>
       <c r="X99" s="131" t="n">
-        <v>629.6630878851374</v>
+        <v>629.6630878851365</v>
       </c>
       <c r="Y99" s="131" t="n">
         <v>23717.12306039543</v>
       </c>
       <c r="Z99" s="132" t="n">
-        <v>32085.23634565483</v>
+        <v>32085.23634565482</v>
       </c>
     </row>
     <row r="100">
@@ -33646,13 +33646,13 @@
         <v>70932</v>
       </c>
       <c r="J104" s="142" t="n">
-        <v>28907.74755960872</v>
+        <v>28907.74755960871</v>
       </c>
       <c r="K104" s="143" t="n">
         <v>13611.05787861222</v>
       </c>
       <c r="L104" s="143" t="n">
-        <v>3961.879579104034</v>
+        <v>3961.879579104033</v>
       </c>
       <c r="M104" s="143" t="n">
         <v>19690.79668663907</v>

</xml_diff>